<commit_message>
Expand FCP sheet workbook to 4 sample ambient products
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RyBLYveiN6TgfgyHKJ8p9M
</commit_message>
<xml_diff>
--- a/FCPシート_商品企画書.xlsx
+++ b/FCPシート_商品企画書.xlsx
@@ -8,10 +8,16 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="FCPシート" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="①ポテトチップス" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="②袋麺" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="③レトルトカレー" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="④ツナ缶" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">FCPシート!$A$1:$H$40</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">①ポテトチップス!$A$1:$H$40</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">②袋麺!$A$1:$H$40</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">③レトルトカレー!$A$1:$H$40</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">④ツナ缶!$A$1:$H$40</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -36,39 +42,73 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">税抜で入力。税込表記が必要な場合は別途注記してください</t>
+          <t xml:space="preserve">税抜で入力。価格・条件は仮の例です。</t>
         </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">(</t>
-        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="B13" authorId="0">
+      <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">消費税率は商品により異なるため自動計算していません</t>
+          <t xml:space="preserve">税抜で入力。価格・条件は仮の例です。</t>
         </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">)</t>
-        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="B13" authorId="0">
+      <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">。</t>
+          <t xml:space="preserve">税抜で入力。価格・条件は仮の例です。</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="B13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">税抜で入力。価格・条件は仮の例です。</t>
         </r>
       </text>
     </comment>
@@ -77,7 +117,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="101">
   <si>
     <r>
       <rPr>
@@ -217,7 +257,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">黄色の欄は記入例です</t>
+      <t xml:space="preserve">黄色の欄は仮の記入例です</t>
     </r>
     <r>
       <rPr>
@@ -236,7 +276,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">上書きして使用</t>
+      <t xml:space="preserve">実際の内容に上書きしてください</t>
     </r>
     <r>
       <rPr>
@@ -327,7 +367,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">4900000000000</t>
+    <t xml:space="preserve">4900000000001</t>
   </si>
   <si>
     <t xml:space="preserve">メーカー・製造元</t>
@@ -828,7 +868,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">個包装ではなく大容量でコストパフォーマンスが高い</t>
+    <t xml:space="preserve">大容量でコストパフォーマンスが高い</t>
   </si>
   <si>
     <r>
@@ -852,7 +892,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">常温で保管でき、バックヤード負担が少ない</t>
+    <t xml:space="preserve">常温保管でバックヤード負担が少ない</t>
   </si>
   <si>
     <r>
@@ -950,14 +990,33 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">棚 〇段目</t>
+      <t xml:space="preserve">棚 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">段目</t>
     </r>
   </si>
   <si>
     <t xml:space="preserve">販売実績・競合比較</t>
   </si>
   <si>
-    <t xml:space="preserve">当店での月間販売数 〇〇個。競合〇〇比で売価−〇円</t>
+    <t xml:space="preserve">当店月間販売数 〇〇個。競合〇〇比で売価−〇円</t>
   </si>
   <si>
     <t xml:space="preserve">販促プラン</t>
@@ -1120,7 +1179,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">右記枠に貼付</t>
+      <t xml:space="preserve">下記枠に貼付</t>
     </r>
     <r>
       <rPr>
@@ -1135,6 +1194,728 @@
   </si>
   <si>
     <t xml:space="preserve">【商品画像貼付エリア】</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〇〇ラーメン 醤油味 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">食パック</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">4900000000002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">〇〇製麺株式会社</t>
+  </si>
+  <si>
+    <t xml:space="preserve">インスタント麺</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">食入</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">食 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100g)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">製造後 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">240</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ケース</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">パック</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">創業以来の定番、あっさり醤油スープ</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">食パックで家庭の買い置きに最適</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">調理時間</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分、アレンジしやすい</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ファミリー層・単身者の常備食</t>
+  </si>
+  <si>
+    <t xml:space="preserve">麺類売場 平台 または 棚 中段</t>
+  </si>
+  <si>
+    <t xml:space="preserve">当店月間販売数 〇〇パック。競合〇〇比で売価−〇円</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">まとめ買い</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">パックで〇〇円、レシピ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">POP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">設置</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〇〇カレー 中辛 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">200g</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">4900000000003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">〇〇フーズ株式会社</t>
+  </si>
+  <si>
+    <t xml:space="preserve">レトルト食品</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">200g(1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">人前</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">製造後 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">720</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ケース</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">受注後 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">営業日</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">国産野菜をじっくり煮込んだコクのある中辛</t>
+  </si>
+  <si>
+    <t xml:space="preserve">湯せん・レンジ対応で手軽</t>
+  </si>
+  <si>
+    <t xml:space="preserve">賞味期限が長く、防災備蓄にも</t>
+  </si>
+  <si>
+    <t xml:space="preserve">共働き世帯・一人暮らし・備蓄ニーズ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">レトルト売場 棚 目線の高さ</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">発売記念で</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個パック販売、試食実施</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〇〇ツナ水煮 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">70g×3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">缶パック</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">4900000000004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">〇〇水産株式会社</t>
+  </si>
+  <si>
+    <t xml:space="preserve">缶詰</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">70g×3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">缶</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">製造後 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1,095</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">タイ</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ケース</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(24</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">パック</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">水煮でヘルシー、サラダや料理に万能</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">缶パックで</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">缶あたりの価格が割安</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">長期保存でき、備蓄にも適する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">健康志向層・調理を楽しむ家庭</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">缶詰売場 棚 中段</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">エンド陳列</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">レシピカード添付、まとめ買い割引</t>
   </si>
 </sst>
 </file>
@@ -1146,7 +1927,7 @@
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1255,11 +2036,6 @@
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1287,12 +2063,25 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -1308,6 +2097,17 @@
       <bottom style="thin">
         <color rgb="FF808080"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -1349,15 +2149,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1365,11 +2165,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1377,15 +2173,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1393,7 +2193,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1714,91 +2514,91 @@
       <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="8" t="s">
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
       <c r="E7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
       <c r="E8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F8" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
       <c r="E9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
       <c r="E10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
@@ -1816,25 +2616,25 @@
       <c r="A13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="9" t="n">
         <v>150</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="9" t="n">
         <v>105</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="4" t="s">
         <v>32</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="10" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1856,11 +2656,11 @@
       <c r="E14" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
@@ -1878,43 +2678,43 @@
       <c r="A17" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
@@ -1932,57 +2732,1620 @@
       <c r="A22" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="14"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
+    </row>
+  </sheetData>
+  <mergeCells count="29">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H30"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A33:H40"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:H40"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="5"/>
+      <c r="F3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>398</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>290</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="11" t="n">
+        <f aca="false">IF(OR(B13="",D13="",B13=0),"",D13/B13)</f>
+        <v>0.728643216080402</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <f aca="false">IF(OR(B13="",D13="",B13=0),"",(B13-D13)/B13)</f>
+        <v>0.271356783919598</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="14"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
+    </row>
+  </sheetData>
+  <mergeCells count="29">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H30"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A33:H40"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:H40"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="5"/>
+      <c r="F3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>178</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="11" t="n">
+        <f aca="false">IF(OR(B13="",D13="",B13=0),"",D13/B13)</f>
+        <v>0.702247191011236</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <f aca="false">IF(OR(B13="",D13="",B13=0),"",(B13-D13)/B13)</f>
+        <v>0.297752808988764</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="14"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
+    </row>
+  </sheetData>
+  <mergeCells count="29">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H30"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A33:H40"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:H40"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="5"/>
+      <c r="F3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>298</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>215</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="11" t="n">
+        <f aca="false">IF(OR(B13="",D13="",B13=0),"",D13/B13)</f>
+        <v>0.721476510067114</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <f aca="false">IF(OR(B13="",D13="",B13=0),"",(B13-D13)/B13)</f>
+        <v>0.278523489932886</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">

</xml_diff>

<commit_message>
Fill FCP sheets with the four actual products and retail prices
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RyBLYveiN6TgfgyHKJ8p9M
</commit_message>
<xml_diff>
--- a/FCPシート_商品企画書.xlsx
+++ b/FCPシート_商品企画書.xlsx
@@ -8,16 +8,16 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="①ポテトチップス" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="②袋麺" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="③レトルトカレー" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="④ツナ缶" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="①柚子ぽん酢" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="②おっさんみそタレ" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="③シンフクロダシ" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="④シンコナコウジ" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">①ポテトチップス!$A$1:$H$40</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">②袋麺!$A$1:$H$40</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">③レトルトカレー!$A$1:$H$40</definedName>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">④ツナ缶!$A$1:$H$40</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">①柚子ぽん酢!$A$1:$H$40</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">②おっさんみそタレ!$A$1:$H$40</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">③シンフクロダシ!$A$1:$H$40</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">④シンコナコウジ!$A$1:$H$40</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -42,7 +42,39 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">税抜で入力。価格・条件は仮の例です。</t>
+          <t xml:space="preserve">税抜で入力。希望小売価格は提示いただいた税別価格。卸価格は未確定のため空欄</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">入力すると掛率・粗利率が計算されます</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">)</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">。</t>
         </r>
       </text>
     </comment>
@@ -64,7 +96,39 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">税抜で入力。価格・条件は仮の例です。</t>
+          <t xml:space="preserve">税抜で入力。希望小売価格は提示いただいた税別価格。卸価格は未確定のため空欄</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">入力すると掛率・粗利率が計算されます</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">)</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">。</t>
         </r>
       </text>
     </comment>
@@ -86,7 +150,39 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">税抜で入力。価格・条件は仮の例です。</t>
+          <t xml:space="preserve">税抜で入力。希望小売価格は提示いただいた税別価格。卸価格は未確定のため空欄</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">入力すると掛率・粗利率が計算されます</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">)</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">。</t>
         </r>
       </text>
     </comment>
@@ -108,7 +204,39 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">税抜で入力。価格・条件は仮の例です。</t>
+          <t xml:space="preserve">税抜で入力。希望小売価格は提示いただいた税別価格。卸価格は未確定のため空欄</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">入力すると掛率・粗利率が計算されます</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">)</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">。</t>
         </r>
       </text>
     </comment>
@@ -117,7 +245,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="46">
   <si>
     <r>
       <rPr>
@@ -257,7 +385,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">黄色の欄は仮の記入例です</t>
+      <t xml:space="preserve">黄色の欄は未確定</t>
     </r>
     <r>
       <rPr>
@@ -276,7 +404,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">実際の内容に上書きしてください</t>
+      <t xml:space="preserve">要記入</t>
     </r>
     <r>
       <rPr>
@@ -295,26 +423,48 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">。</t>
+      <t xml:space="preserve">の欄です。</t>
     </r>
   </si>
   <si>
     <t xml:space="preserve">商談日</t>
   </si>
   <si>
-    <t xml:space="preserve">2026/11/01</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">要記入</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">提案先</t>
   </si>
   <si>
-    <t xml:space="preserve">〇〇株式会社 ご担当者様</t>
-  </si>
-  <si>
     <t xml:space="preserve">提案者</t>
-  </si>
-  <si>
-    <t xml:space="preserve">当店 〇〇</t>
   </si>
   <si>
     <r>
@@ -343,7 +493,7 @@
     <t xml:space="preserve">商品名</t>
   </si>
   <si>
-    <t xml:space="preserve">〇〇ポテトチップス うすしお</t>
+    <t xml:space="preserve">幻の柚子 実生の柚子ぽん酢</t>
   </si>
   <si>
     <r>
@@ -367,27 +517,55 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">4900000000001</t>
-  </si>
-  <si>
     <t xml:space="preserve">メーカー・製造元</t>
   </si>
   <si>
-    <t xml:space="preserve">〇〇食品株式会社</t>
-  </si>
-  <si>
     <t xml:space="preserve">カテゴリ</t>
   </si>
   <si>
-    <t xml:space="preserve">スナック菓子</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">調味料</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ぽん酢</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">規格・内容量</t>
   </si>
   <si>
-    <t xml:space="preserve">60g</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -474,92 +652,56 @@
     <t xml:space="preserve">賞味期限</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">製造後 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">180</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
+    <t xml:space="preserve">原産国</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">発売</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">予定</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">日</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">原産国</t>
-  </si>
-  <si>
-    <t xml:space="preserve">日本</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">発売</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">予定</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/12/01</t>
   </si>
   <si>
     <r>
@@ -668,48 +810,44 @@
     <t xml:space="preserve">最低発注ロット</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ケース</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(24</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
+    <t xml:space="preserve">納期</t>
+  </si>
+  <si>
+    <t xml:space="preserve">掛率</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">想定粗利率</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">売価ベース</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -718,86 +856,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">納期</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">受注後 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">営業日</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">掛率</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">想定粗利率</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">売価ベース</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">支払条件</t>
-  </si>
-  <si>
-    <t xml:space="preserve">月末締め翌月末払い</t>
   </si>
   <si>
     <r>
@@ -844,9 +903,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">素材にこだわった、軽い食感のうすしお味</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -868,9 +924,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">大容量でコストパフォーマンスが高い</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -890,9 +943,6 @@
       </rPr>
       <t xml:space="preserve">3</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">常温保管でバックヤード負担が少ない</t>
   </si>
   <si>
     <r>
@@ -921,154 +971,13 @@
     <t xml:space="preserve">ターゲット顧客</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">〜</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">代の家庭向け・買い置き需要</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">提案売場・陳列</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">菓子売場 エンド陳列</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">棚 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">段目</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">販売実績・競合比較</t>
   </si>
   <si>
-    <t xml:space="preserve">当店月間販売数 〇〇個。競合〇〇比で売価−〇円</t>
-  </si>
-  <si>
     <t xml:space="preserve">販促プラン</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">発売</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">週間は特売価格〇〇円、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">POP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・試食実施</t>
-    </r>
   </si>
   <si>
     <r>
@@ -1096,8 +1005,63 @@
   <si>
     <r>
       <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">商品画像</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">下記枠に貼付</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">【商品画像貼付エリア】</t>
+  </si>
+  <si>
+    <t xml:space="preserve">青とうがらし焼肉おっさんみそタレ</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
         <sz val="10"/>
         <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">調味料</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -1111,7 +1075,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">例</t>
+      <t xml:space="preserve">焼肉のタレ</t>
     </r>
     <r>
       <rPr>
@@ -1123,6 +1087,8 @@
       </rPr>
       <t xml:space="preserve">)</t>
     </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="10"/>
@@ -1130,7 +1096,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">サンプル提供のお願い</t>
+      <t xml:space="preserve">袋だし </t>
     </r>
     <r>
       <rPr>
@@ -1140,7 +1106,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">/</t>
+      <t xml:space="preserve">[</t>
     </r>
     <r>
       <rPr>
@@ -1149,773 +1115,64 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">ケース規格・パレット積付けの確認 など</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">商品画像</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">下記枠に貼付</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">【商品画像貼付エリア】</t>
-  </si>
-  <si>
+      <t xml:space="preserve">シンフクロダシ</t>
+    </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">〇〇ラーメン 醤油味 </t>
-    </r>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">だし</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">粉糀 </t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">食パック</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">4900000000002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">〇〇製麺株式会社</t>
-  </si>
-  <si>
-    <t xml:space="preserve">インスタント麺</t>
-  </si>
-  <si>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[</t>
+    </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">シンコナコウジ</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">食入</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">食 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100g)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">製造後 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">240</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ケース</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(6</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">パック</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">創業以来の定番、あっさり醤油スープ</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">食パックで家庭の買い置きに最適</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">調理時間</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">分、アレンジしやすい</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">ファミリー層・単身者の常備食</t>
-  </si>
-  <si>
-    <t xml:space="preserve">麺類売場 平台 または 棚 中段</t>
-  </si>
-  <si>
-    <t xml:space="preserve">当店月間販売数 〇〇パック。競合〇〇比で売価−〇円</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">まとめ買い</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">パックで〇〇円、レシピ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">POP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">設置</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">〇〇カレー 中辛 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">200g</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">4900000000003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">〇〇フーズ株式会社</t>
-  </si>
-  <si>
-    <t xml:space="preserve">レトルト食品</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">200g(1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">人前</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">製造後 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">720</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ケース</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(30</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">受注後 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">営業日</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">国産野菜をじっくり煮込んだコクのある中辛</t>
-  </si>
-  <si>
-    <t xml:space="preserve">湯せん・レンジ対応で手軽</t>
-  </si>
-  <si>
-    <t xml:space="preserve">賞味期限が長く、防災備蓄にも</t>
-  </si>
-  <si>
-    <t xml:space="preserve">共働き世帯・一人暮らし・備蓄ニーズ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">レトルト売場 棚 目線の高さ</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">発売記念で</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個パック販売、試食実施</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">〇〇ツナ水煮 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">70g×3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">缶パック</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">4900000000004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">〇〇水産株式会社</t>
-  </si>
-  <si>
-    <t xml:space="preserve">缶詰</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">70g×3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">缶</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">製造後 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1,095</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">タイ</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ケース</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(24</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">パック</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">水煮でヘルシー、サラダや料理に万能</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">缶パックで</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">缶あたりの価格が割安</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">長期保存でき、備蓄にも適する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">健康志向層・調理を楽しむ家庭</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">缶詰売場 棚 中段</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">エンド陳列</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">レシピカード添付、まとめ買い割引</t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">糀</t>
   </si>
 </sst>
 </file>
@@ -1927,7 +1184,7 @@
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2034,6 +1291,11 @@
     <font>
       <sz val="10"/>
       <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -2157,7 +1419,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2165,19 +1427,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2487,20 +1749,20 @@
         <v>4</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H3" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -2512,97 +1774,97 @@
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
+      <c r="F6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+        <v>11</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
+        <v>13</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
       <c r="E8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
+        <v>14</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
       <c r="E9" s="3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
+        <v>19</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -2614,57 +1876,55 @@
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B13" s="9" t="n">
-        <v>150</v>
+        <v>1300</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>105</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="D13" s="10"/>
       <c r="E13" s="3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>34</v>
+        <v>24</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="B14" s="11" t="str">
         <f aca="false">IF(OR(B13="",D13="",B13=0),"",D13/B13)</f>
-        <v>0.7</v>
+        <v/>
       </c>
       <c r="C14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D14" s="11" t="str">
         <f aca="false">IF(OR(B13="",D13="",B13=0),"",(B13-D13)/B13)</f>
-        <v>0.3</v>
+        <v/>
       </c>
       <c r="E14" s="3" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -2676,10 +1936,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -2690,10 +1950,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -2704,10 +1964,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -2718,7 +1978,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -2730,24 +1990,24 @@
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
+        <v>33</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -2758,10 +2018,10 @@
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
@@ -2772,10 +2032,10 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>54</v>
+        <v>3</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
@@ -2786,7 +2046,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -2798,7 +2058,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="B28" s="12"/>
       <c r="C28" s="12"/>
@@ -2830,7 +2090,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
@@ -2842,7 +2102,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -3008,20 +2268,20 @@
         <v>4</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H3" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -3033,97 +2293,97 @@
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
+      <c r="F6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+        <v>11</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
+        <v>13</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
       <c r="E8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
+        <v>14</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
       <c r="E9" s="3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>64</v>
+        <v>3</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
+        <v>19</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -3135,57 +2395,55 @@
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B13" s="9" t="n">
-        <v>398</v>
+        <v>1300</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>290</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="D13" s="10"/>
       <c r="E13" s="3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>34</v>
+        <v>24</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="B14" s="11" t="str">
         <f aca="false">IF(OR(B13="",D13="",B13=0),"",D13/B13)</f>
-        <v>0.728643216080402</v>
+        <v/>
       </c>
       <c r="C14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D14" s="11" t="str">
         <f aca="false">IF(OR(B13="",D13="",B13=0),"",(B13-D13)/B13)</f>
-        <v>0.271356783919598</v>
+        <v/>
       </c>
       <c r="E14" s="3" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -3197,10 +2455,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>66</v>
+        <v>3</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -3211,24 +2469,24 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
+        <v>30</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -3239,7 +2497,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -3251,10 +2509,10 @@
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>69</v>
+        <v>3</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
@@ -3265,10 +2523,10 @@
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -3279,10 +2537,10 @@
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
@@ -3293,10 +2551,10 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>72</v>
+        <v>3</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
@@ -3307,7 +2565,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -3319,7 +2577,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="B28" s="12"/>
       <c r="C28" s="12"/>
@@ -3351,7 +2609,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
@@ -3363,7 +2621,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -3529,20 +2787,20 @@
         <v>4</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H3" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -3554,97 +2812,97 @@
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
+      <c r="F6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>75</v>
+        <v>3</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+        <v>11</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
+        <v>13</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
       <c r="E8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
+        <v>14</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
       <c r="E9" s="3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>78</v>
+        <v>3</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
+        <v>19</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -3656,57 +2914,55 @@
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B13" s="9" t="n">
-        <v>178</v>
+        <v>2000</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>125</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="D13" s="10"/>
       <c r="E13" s="3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>79</v>
+        <v>3</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>80</v>
+        <v>24</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="B14" s="11" t="str">
         <f aca="false">IF(OR(B13="",D13="",B13=0),"",D13/B13)</f>
-        <v>0.702247191011236</v>
+        <v/>
       </c>
       <c r="C14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D14" s="11" t="str">
         <f aca="false">IF(OR(B13="",D13="",B13=0),"",(B13-D13)/B13)</f>
-        <v>0.297752808988764</v>
+        <v/>
       </c>
       <c r="E14" s="3" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -3718,10 +2974,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>81</v>
+        <v>3</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -3732,10 +2988,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>82</v>
+        <v>3</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -3746,10 +3002,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>83</v>
+        <v>3</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -3760,7 +3016,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -3772,10 +3028,10 @@
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>84</v>
+        <v>3</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
@@ -3786,10 +3042,10 @@
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>85</v>
+        <v>3</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -3800,10 +3056,10 @@
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
@@ -3814,10 +3070,10 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>86</v>
+        <v>3</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
@@ -3828,7 +3084,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -3840,7 +3096,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="B28" s="12"/>
       <c r="C28" s="12"/>
@@ -3872,7 +3128,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
@@ -3884,7 +3140,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -4050,20 +3306,20 @@
         <v>4</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H3" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -4075,97 +3331,97 @@
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
+      <c r="F6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>89</v>
+        <v>3</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+        <v>11</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
+        <v>13</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
       <c r="E8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
+        <v>14</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
       <c r="E9" s="3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>92</v>
+        <v>3</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>93</v>
+        <v>3</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
+        <v>19</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -4177,57 +3433,55 @@
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B13" s="9" t="n">
-        <v>298</v>
+        <v>2000</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>215</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="D13" s="10"/>
       <c r="E13" s="3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>94</v>
+        <v>3</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>80</v>
+        <v>24</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="B14" s="11" t="str">
         <f aca="false">IF(OR(B13="",D13="",B13=0),"",D13/B13)</f>
-        <v>0.721476510067114</v>
+        <v/>
       </c>
       <c r="C14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D14" s="11" t="str">
         <f aca="false">IF(OR(B13="",D13="",B13=0),"",(B13-D13)/B13)</f>
-        <v>0.278523489932886</v>
+        <v/>
       </c>
       <c r="E14" s="3" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -4239,10 +3493,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -4253,24 +3507,24 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
+        <v>30</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -4281,7 +3535,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -4293,10 +3547,10 @@
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>98</v>
+        <v>3</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
@@ -4307,10 +3561,10 @@
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>99</v>
+        <v>3</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -4321,10 +3575,10 @@
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
@@ -4335,10 +3589,10 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
@@ -4349,7 +3603,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -4361,7 +3615,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="B28" s="12"/>
       <c r="C28" s="12"/>
@@ -4393,7 +3647,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
@@ -4405,7 +3659,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>

</xml_diff>

<commit_message>
Embed shop logo in each FCP sheet header
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RyBLYveiN6TgfgyHKJ8p9M
</commit_message>
<xml_diff>
--- a/FCPシート_商品企画書.xlsx
+++ b/FCPシート_商品企画書.xlsx
@@ -1531,6 +1531,174 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>590040</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>47160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8176320" y="0"/>
+          <a:ext cx="590040" cy="599760"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>590040</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>47160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8176320" y="0"/>
+          <a:ext cx="590040" cy="599760"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>590040</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>47160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8176320" y="0"/>
+          <a:ext cx="590040" cy="599760"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>590040</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>47160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8176320" y="0"/>
+          <a:ext cx="590040" cy="599760"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -1721,7 +1889,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1731,9 +1899,8 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2184,7 +2351,7 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="A5:H5"/>
@@ -2221,7 +2388,8 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -2240,7 +2408,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2250,9 +2418,8 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2703,7 +2870,7 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="A5:H5"/>
@@ -2740,7 +2907,8 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -2759,7 +2927,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2769,9 +2937,8 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -3222,7 +3389,7 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="A5:H5"/>
@@ -3259,7 +3426,8 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -3278,7 +3446,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3288,9 +3456,8 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -3741,7 +3908,7 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="A5:H5"/>
@@ -3778,6 +3945,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add product photo and package info to FCP sheet 4
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RyBLYveiN6TgfgyHKJ8p9M
</commit_message>
<xml_diff>
--- a/FCPシート_商品企画書.xlsx
+++ b/FCPシート_商品企画書.xlsx
@@ -245,7 +245,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="51">
   <si>
     <r>
       <rPr>
@@ -1172,7 +1172,151 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">畑名味噌糀店</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">四国阿波勝浦</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">糀</t>
+  </si>
+  <si>
+    <t xml:space="preserve">石臼挽き仕立て。より低温で、より細かく挽いた粉糀</t>
+  </si>
+  <si>
+    <t xml:space="preserve">料理にサッと一振りするだけで、お手軽に酵素生活</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">創業明治</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年、四国阿波勝浦の糀店が手がける粉糀</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">創業 明治</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">パッケージ記載</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。商品写真はパッケージ現物。</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1398,7 +1542,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1457,6 +1601,14 @@
     </xf>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1696,6 +1848,43 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>957960</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>380880</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3524400" y="8096400"/>
+          <a:ext cx="2085480" cy="3714480"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3518,16 +3707,16 @@
       <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
+      <c r="B7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
@@ -3662,43 +3851,43 @@
       <c r="A17" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
+      <c r="B17" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
+      <c r="B18" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
+      <c r="B19" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
@@ -3781,36 +3970,36 @@
       <c r="H27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
+      <c r="A28" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
+      <c r="A29" s="15"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="12"/>
+      <c r="A30" s="15"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
@@ -3824,87 +4013,85 @@
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="14"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="14"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="14"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="14"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="14"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="14"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
+    <row r="33" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="16"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="16"/>
+    </row>
+    <row r="34" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="16"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16"/>
+      <c r="H34" s="16"/>
+    </row>
+    <row r="35" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="16"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="16"/>
+    </row>
+    <row r="36" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="16"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
+    </row>
+    <row r="37" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="16"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+    </row>
+    <row r="38" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="16"/>
+      <c r="B38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="16"/>
+      <c r="H38" s="16"/>
+    </row>
+    <row r="39" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="16"/>
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="16"/>
+    </row>
+    <row r="40" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="16"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="29">

</xml_diff>